<commit_message>
update branch w new colors
</commit_message>
<xml_diff>
--- a/statistical_analyses/rsu_ensemble.xlsx
+++ b/statistical_analyses/rsu_ensemble.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brynr/Desktop/SPECTRA_evaluation/statistical_analyses/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C669502A-05C2-784A-97CA-5C2B4D8E92DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{552DCFE5-82D5-3945-93AE-6A611D2D88C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36180" yWindow="2380" windowWidth="28800" windowHeight="17220" activeTab="10" xr2:uid="{552454A9-BAD3-2547-BBF5-703F9608AD65}"/>
+    <workbookView xWindow="36980" yWindow="3860" windowWidth="28800" windowHeight="17220" activeTab="10" xr2:uid="{552454A9-BAD3-2547-BBF5-703F9608AD65}"/>
   </bookViews>
   <sheets>
     <sheet name="bace" sheetId="2" r:id="rId1"/>
@@ -22,12 +22,13 @@
     <sheet name="sider" sheetId="7" r:id="rId7"/>
     <sheet name="tox21" sheetId="8" r:id="rId8"/>
     <sheet name="summary" sheetId="9" r:id="rId9"/>
-    <sheet name="machine_readable" sheetId="10" r:id="rId10"/>
-    <sheet name="baselines_mr" sheetId="11" r:id="rId11"/>
+    <sheet name="spectra_results" sheetId="12" r:id="rId10"/>
+    <sheet name="random_scaffold_umap" sheetId="10" r:id="rId11"/>
+    <sheet name="classical_baselines" sheetId="11" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="baselines2" localSheetId="10">baselines_mr!$A$93:$G$213</definedName>
-    <definedName name="linear_baseline_results" localSheetId="10">baselines_mr!$A$1:$E$91</definedName>
+    <definedName name="baselines2" localSheetId="11">classical_baselines!$A$93:$G$213</definedName>
+    <definedName name="linear_baseline_results" localSheetId="11">classical_baselines!$A$1:$E$91</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -52,7 +53,7 @@
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
 <connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16">
   <connection id="1" xr16:uid="{466AD2AA-DDFD-0847-8256-11220658BF06}" name="baselines2" type="6" refreshedVersion="8" background="1" saveData="1">
-    <textPr codePage="10000" sourceFile="/Users/brynr/Desktop/SPECTRA_evaluation/statistical_analyses/baselines2.csv" comma="1">
+    <textPr sourceFile="/Users/brynr/Desktop/SPECTRA_evaluation/statistical_analyses/baselines2.csv" comma="1">
       <textFields count="7">
         <textField/>
         <textField/>
@@ -11448,6 +11449,15 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA8824F9-334B-E44D-B50A-5773C289CA0A}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F9C84EFF-0C96-EE4D-962D-099FC06205CE}">
   <dimension ref="A1:X201"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -17815,7 +17825,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B78A611-F410-5048-B748-F0E63A286AE3}">
   <dimension ref="A1:E211"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>